<commit_message>
use rdp in opacus
</commit_message>
<xml_diff>
--- a/cnn results/cnn result.xlsx
+++ b/cnn results/cnn result.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\flight delay\stpn paper\STPN-main\cnn results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895A3241-2FAF-447E-80BA-D8893990B2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801516EC-A020-4718-8824-9CCB064796A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="time" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="time" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="44">
   <si>
     <t>sigma</t>
   </si>
@@ -98,6 +99,66 @@
   </si>
   <si>
     <t>15763 opacus_udata_cnn_dp_three_stage_summary_sigma2_00_20260110_202933.csv​</t>
+  </si>
+  <si>
+    <t>Run ID / Description</t>
+  </si>
+  <si>
+    <t>Dataset (train / val / test)</t>
+  </si>
+  <si>
+    <t>Sigma (noise multiplier)</t>
+  </si>
+  <si>
+    <t>Target ε</t>
+  </si>
+  <si>
+    <t>Final ε</t>
+  </si>
+  <si>
+    <t>Classification F1 (macro)</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>MAE delayed (min)</t>
+  </si>
+  <si>
+    <t>MAE non-delayed (min)</t>
+  </si>
+  <si>
+    <t>MAE overall (min)</t>
+  </si>
+  <si>
+    <t>csv summary (three-stage, large cdata)</t>
+  </si>
+  <si>
+    <t>55,218 / 7,871 / 15,763</t>
+  </si>
+  <si>
+    <t>1.00 (from filename)</t>
+  </si>
+  <si>
+    <t>run 20260110-19:39:46 (cdatasigma0.50)</t>
+  </si>
+  <si>
+    <t>19,207 / 2,727 / 5,474</t>
+  </si>
+  <si>
+    <t>run 20260110-19:42:23 (cdatasigma0.50, repeat)</t>
+  </si>
+  <si>
+    <t>run 20260110-19:39:58 (cdatasigma1.00)</t>
+  </si>
+  <si>
+    <t>opacus udata</t>
+  </si>
+  <si>
+    <t>non opacus udata</t>
+  </si>
+  <si>
+    <t>cdata opacus</t>
   </si>
 </sst>
 </file>
@@ -146,7 +207,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -169,11 +230,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -185,6 +266,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,14 +557,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
     <col min="8" max="14" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="24.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="24.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -502,8 +592,11 @@
       <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K1" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -532,7 +625,7 @@
         <v>0.95138285007312295</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -561,136 +654,304 @@
         <v>0.50164456508782196</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="1:14" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="11" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="2">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2">
+        <v>3.0579999999999998</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.54600000000000004</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.71589999999999998</v>
+      </c>
+      <c r="H12" s="2">
+        <v>8.4255999999999993</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4.8490000000000002</v>
+      </c>
+      <c r="J12" s="2">
+        <v>5.7145000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="2">
+        <v>11</v>
+      </c>
+      <c r="E13" s="2">
+        <v>2.9449999999999998</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.54359999999999997</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.71360000000000001</v>
+      </c>
+      <c r="H13" s="2">
+        <v>8.4669000000000008</v>
+      </c>
+      <c r="I13" s="2">
+        <v>4.7637</v>
+      </c>
+      <c r="J13" s="2">
+        <v>5.6597999999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6">
+        <f>AVERAGE(C12:C13)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="6">
+        <f>AVERAGE(D12:D13)</f>
+        <v>11</v>
+      </c>
+      <c r="E14" s="6">
+        <f>AVERAGE(E12:E13)</f>
+        <v>3.0015000000000001</v>
+      </c>
+      <c r="F14" s="6">
+        <f>AVERAGE(F12:F13)</f>
+        <v>0.54479999999999995</v>
+      </c>
+      <c r="G14" s="6">
+        <f>AVERAGE(G12:G13)</f>
+        <v>0.71475</v>
+      </c>
+      <c r="H14" s="6">
+        <f>AVERAGE(H12:H13)</f>
+        <v>8.4462499999999991</v>
+      </c>
+      <c r="I14" s="6">
+        <f>AVERAGE(I12:I13)</f>
+        <v>4.8063500000000001</v>
+      </c>
+      <c r="J14" s="6">
+        <f>AVERAGE(J12:J13)</f>
+        <v>5.6871499999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6">
+        <v>11</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0.51080000000000003</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0.71840000000000004</v>
+      </c>
+      <c r="H15" s="6">
+        <v>8.8719000000000001</v>
+      </c>
+      <c r="I15" s="6">
+        <v>4.6685999999999996</v>
+      </c>
+      <c r="J15" s="6">
+        <v>5.6856999999999998</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="71" spans="1:14" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B71" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D71" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F71" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G71" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H71" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I71" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J71" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K71" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L71" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M71" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="N71" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2">
+    <row r="72" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B72" s="2">
         <v>0.44367262209337399</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C72" s="2">
         <v>1.46259770652995E-2</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D72" s="2">
         <v>2.82764220013264E-2</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E72" s="2">
         <v>0.81599541421592303</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F72" s="2">
         <v>12.310812756096301</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G72" s="2">
         <v>14.577960783877099</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H72" s="2">
         <v>0.95138285007312295</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I72" s="2">
         <v>1.45057793488848</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J72" s="2">
         <v>3.03402392662086</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K72" s="2">
         <v>6.37819032139575</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L72" s="2">
         <v>404599</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M72" s="2">
         <v>1802221</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N72" s="2">
         <v>0.12813553514614001</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2">
+    <row r="73" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="2">
         <v>2</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B73" s="2">
         <v>0.26816671281738003</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C73" s="2">
         <v>1.1342648985602399E-3</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D73" s="2">
         <v>2.2580678749840001E-3</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E73" s="2">
         <v>0.81654416762580695</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F73" s="2">
         <v>13.375944175026399</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G73" s="2">
         <v>15.473525828896999</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H73" s="2">
         <v>0.50164456508782196</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I73" s="2">
         <v>0.99998352736971297</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J73" s="2">
         <v>2.8620222795736101</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K73" s="2">
         <v>6.6868375709511803</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L73" s="2">
         <v>404599</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M73" s="2">
         <v>1802221</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N73" s="2">
         <v>5.3868287199408497E-2</v>
       </c>
     </row>
@@ -701,6 +962,83 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8CC8DD-ACC4-41BB-82CE-4167213D5E66}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:12" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="83.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="2">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2">
+        <v>101.42</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.36109999999999998</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0.63029999999999997</v>
+      </c>
+      <c r="H2" s="2">
+        <v>7.4020000000000001</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3.7728000000000002</v>
+      </c>
+      <c r="J2" s="2">
+        <v>6.2095000000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD62EE0-B23C-4003-BB7F-31D7884A295E}">
   <dimension ref="B1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>